<commit_message>
feat: Implement Modules Variável, Benefícios, Apontamentos and Report Versioning
</commit_message>
<xml_diff>
--- a/templates/02. Templeta_ 2025 FOLHA DE PAGAMENTO - SUPER INDUSTRIA & CAFFEINE ARMY.xlsx
+++ b/templates/02. Templeta_ 2025 FOLHA DE PAGAMENTO - SUPER INDUSTRIA & CAFFEINE ARMY.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo.rodrigues\Documents\Rodrigues\11. Automação Google Sheets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{374DD743-5B50-42B8-BA9F-3F17BB42FC81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1550ED05-0F80-468F-A96E-E5D55CBCA2CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Página14" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Filtro 2" guid="{B3412BFF-8E92-4B96-9B14-EBC15F534955}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Filtro 1" guid="{2F83DE60-6623-4425-8959-D7FAD0F01E57}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 2" guid="{B3412BFF-8E92-4B96-9B14-EBC15F534955}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>8111 (AMIL 2)</t>
   </si>
@@ -682,21 +682,31 @@
         <v>37122</v>
       </c>
       <c r="K3" s="13">
-        <f t="shared" ref="K3:K5" ca="1" si="0">DATEDIF(J3,TODAY(),"Y")</f>
+        <f ca="1">DATEDIF($J3,TODAY(),"Y")</f>
         <v>24</v>
       </c>
-      <c r="L3" s="22" t="s">
-        <v>22</v>
+      <c r="L3" s="22" t="str">
+        <f ca="1">IF($K3&lt;=18,"0-18",
+IF($K3&lt;=23,"19-23",
+IF($K3&lt;=28,"24-28",
+IF($K3&lt;=33,"29-33",
+IF($K3&lt;=38,"34-38",
+IF($K3&lt;=43,"39-43",
+IF($K3&lt;=48,"44-48",
+IF($K3&lt;=53,"49-53",
+IF($K3&lt;=58,"54-58","59 ou mais"
+)))))))))</f>
+        <v>24-28</v>
       </c>
       <c r="M3" s="15">
         <v>0</v>
       </c>
       <c r="N3" s="15">
-        <f t="shared" ref="N3:N5" si="1">M3*80%</f>
+        <f t="shared" ref="N3:N5" si="0">M3*80%</f>
         <v>0</v>
       </c>
       <c r="O3" s="16">
-        <f t="shared" ref="O3:O5" si="2">M3*20%</f>
+        <f t="shared" ref="O3:O5" si="1">M3*20%</f>
         <v>0</v>
       </c>
       <c r="P3" s="16">
@@ -737,21 +747,31 @@
         <v>37773</v>
       </c>
       <c r="K4" s="13">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ref="K3:K5" ca="1" si="2">DATEDIF(J4,TODAY(),"Y")</f>
         <v>22</v>
       </c>
-      <c r="L4" s="22" t="s">
-        <v>22</v>
+      <c r="L4" s="22" t="str">
+        <f t="shared" ref="L4:L5" ca="1" si="3">IF($K4&lt;=18,"0-18",
+IF($K4&lt;=23,"19-23",
+IF($K4&lt;=28,"24-28",
+IF($K4&lt;=33,"29-33",
+IF($K4&lt;=38,"34-38",
+IF($K4&lt;=43,"39-43",
+IF($K4&lt;=48,"44-48",
+IF($K4&lt;=53,"49-53",
+IF($K4&lt;=58,"54-58","59 ou mais"
+)))))))))</f>
+        <v>19-23</v>
       </c>
       <c r="M4" s="15">
         <v>0</v>
       </c>
       <c r="N4" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O4" s="16">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O4" s="16">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P4" s="16">
@@ -792,19 +812,22 @@
         <v>33330</v>
       </c>
       <c r="K5" s="13">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="2"/>
         <v>34</v>
       </c>
-      <c r="L5" s="14"/>
+      <c r="L5" s="14" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>34-38</v>
+      </c>
       <c r="M5" s="15">
         <v>0</v>
       </c>
       <c r="N5" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="16">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O5" s="16">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P5" s="16">

</xml_diff>

<commit_message>
fix: update calculation logic for health plans and gas integration
</commit_message>
<xml_diff>
--- a/templates/02. Templeta_ 2025 FOLHA DE PAGAMENTO - SUPER INDUSTRIA & CAFFEINE ARMY.xlsx
+++ b/templates/02. Templeta_ 2025 FOLHA DE PAGAMENTO - SUPER INDUSTRIA & CAFFEINE ARMY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo.rodrigues\Documents\Rodrigues\11. Automação Google Sheets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1550ED05-0F80-468F-A96E-E5D55CBCA2CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5561CEFB-F8D3-43F0-A8D7-5132F31F5D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Página14" sheetId="2" r:id="rId1"/>
@@ -37,19 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
-  <si>
-    <t>8111 (AMIL 2)</t>
-  </si>
-  <si>
-    <t>313 (AMIL 2)</t>
-  </si>
-  <si>
-    <t>370 (AMIL ODONTO 13)</t>
-  </si>
-  <si>
-    <t>392 (AMIL ODONTO 13)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="56">
   <si>
     <t>NOME</t>
   </si>
@@ -66,9 +54,6 @@
     <t>SALÁRIO</t>
   </si>
   <si>
-    <t>NOVO SALÁRIO</t>
-  </si>
-  <si>
     <t>CARGO</t>
   </si>
   <si>
@@ -123,29 +108,114 @@
     <t>PRODUTOS</t>
   </si>
   <si>
-    <t>ANALISTA COMERCIAL PLENO</t>
-  </si>
-  <si>
-    <t>B2B GESTÃO DE CARTEIRA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANA </t>
-  </si>
-  <si>
-    <t>BIA</t>
-  </si>
-  <si>
-    <t>JOÃO</t>
+    <t>ALICE BASTOS CAMPOS</t>
+  </si>
+  <si>
+    <t>Filial Ba</t>
+  </si>
+  <si>
+    <t>COPYWRITER PLENO</t>
+  </si>
+  <si>
+    <t>GERAL</t>
+  </si>
+  <si>
+    <t>AMIL S580 QP NAC R PJ</t>
+  </si>
+  <si>
+    <t>29-33</t>
+  </si>
+  <si>
+    <t>ALICE PEREIRA MOREIRA DE OLIVEIRA NETA</t>
+  </si>
+  <si>
+    <t>ESTAGIÁRIO DE FINANCEIRO</t>
+  </si>
+  <si>
+    <t>FINANCEIRO</t>
+  </si>
+  <si>
+    <t>ALINE SOUZA BARROSO SANTOS</t>
+  </si>
+  <si>
+    <t>ANALISTA DE T.I JUNIOR</t>
+  </si>
+  <si>
+    <t>TECNOLOGIA</t>
+  </si>
+  <si>
+    <t>AMIL S750 R2 QP NAC PJ</t>
+  </si>
+  <si>
+    <t>24-28</t>
+  </si>
+  <si>
+    <t>ALLAN RODRIGO GOMES COSTA</t>
+  </si>
+  <si>
+    <t>ANALISTA DE INTELIGENCIA COMERCIAL PLENO</t>
+  </si>
+  <si>
+    <t>B2B</t>
+  </si>
+  <si>
+    <t>R$ 24,24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMANDA BORGES CORDEIRO CARNEIRO </t>
+  </si>
+  <si>
+    <t>COORDENADOR DE GROWTH</t>
+  </si>
+  <si>
+    <t>B2C</t>
+  </si>
+  <si>
+    <t>AMANDA DE JESUS PAIXAO</t>
+  </si>
+  <si>
+    <t>ANALISTA SOCIAL MEDIA JUNIOR</t>
+  </si>
+  <si>
+    <t>SOCIAL STRATEGY</t>
+  </si>
+  <si>
+    <t>ANA BEATRIZ BRANDÃO SOARES</t>
+  </si>
+  <si>
+    <t>ESTAGIÁRIO TRADE MARKETING</t>
+  </si>
+  <si>
+    <t>ANA CAROLINA MEKITARIAN NUNES</t>
+  </si>
+  <si>
+    <t>ANA LAURA BONFIM ESTEVES</t>
+  </si>
+  <si>
+    <t>Status (Pendente/Pago)</t>
+  </si>
+  <si>
+    <t>Data Pagto</t>
+  </si>
+  <si>
+    <t>Obs</t>
+  </si>
+  <si>
+    <t>PAGO</t>
+  </si>
+  <si>
+    <t>SÓCIO: ADIANTAMENTO DE LUCRO - VALOR R$ 15.000,00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$R$ -416]#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -185,6 +255,27 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -212,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -246,18 +337,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -270,15 +383,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -330,8 +437,21 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -548,297 +668,630 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="53.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="2"/>
       <c r="H1" s="3"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
       <c r="N1" s="4"/>
-      <c r="O1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="P1" s="5" t="s">
+      <c r="O1" s="4"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+    </row>
+    <row r="2" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="G2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="H2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="J2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="K2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="L2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="M2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="N2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="O2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="P2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="Q2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="R2" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="S2" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="T2" s="31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="16">
+        <v>45231</v>
+      </c>
+      <c r="D3" s="16"/>
+      <c r="E3" s="18">
+        <v>11344.708154521117</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="9">
+        <v>34595</v>
+      </c>
+      <c r="J3" s="10">
+        <v>31</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" s="12">
+        <v>984.21</v>
+      </c>
+      <c r="M3" s="12">
+        <v>787.36800000000005</v>
+      </c>
+      <c r="N3" s="13">
+        <v>196.84200000000001</v>
+      </c>
+      <c r="O3" s="13">
+        <v>0</v>
+      </c>
+      <c r="P3" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="27">
+        <v>0</v>
+      </c>
+      <c r="R3" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="30">
+        <v>45672</v>
+      </c>
+      <c r="T3" s="29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="16">
+        <v>45950</v>
+      </c>
+      <c r="D4" s="16"/>
+      <c r="E4" s="18">
+        <v>12641.453555310802</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="I4" s="9">
+        <v>36274</v>
+      </c>
+      <c r="J4" s="10">
+        <v>26</v>
+      </c>
+      <c r="K4" s="19"/>
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+      <c r="M4" s="12">
+        <v>0</v>
+      </c>
+      <c r="N4" s="13">
+        <v>0</v>
+      </c>
+      <c r="O4" s="13">
+        <v>0</v>
+      </c>
+      <c r="P4" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="27">
+        <v>0</v>
+      </c>
+      <c r="R4" s="28"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="28"/>
+    </row>
+    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="22">
+        <v>45880</v>
+      </c>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23">
+        <v>8784.0854450045481</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="9">
+        <v>35952</v>
+      </c>
+      <c r="J5" s="10">
+        <v>27</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="12">
+        <v>941.13</v>
+      </c>
+      <c r="M5" s="12">
+        <v>752.904</v>
+      </c>
+      <c r="N5" s="13">
+        <v>188.226</v>
+      </c>
+      <c r="O5" s="13">
+        <v>0</v>
+      </c>
+      <c r="P5" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="27">
+        <v>0</v>
+      </c>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+    </row>
+    <row r="6" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="16">
+        <v>45566</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="18">
+        <v>9793.091342551148</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="9">
+        <v>33653</v>
+      </c>
+      <c r="J6" s="10">
+        <v>33</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="12">
+        <v>984.21</v>
+      </c>
+      <c r="M6" s="12">
+        <v>787.36800000000005</v>
+      </c>
+      <c r="N6" s="13">
+        <v>196.84200000000001</v>
+      </c>
+      <c r="O6" s="13">
+        <v>0</v>
+      </c>
+      <c r="P6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" s="27">
+        <v>0</v>
+      </c>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="28"/>
+    </row>
+    <row r="7" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="16">
+        <v>45698</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="18">
+        <v>10925.752087042414</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="9">
+        <v>35709</v>
+      </c>
+      <c r="J7" s="10">
+        <v>28</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="L7" s="12">
+        <v>941.13</v>
+      </c>
+      <c r="M7" s="12">
+        <v>752.904</v>
+      </c>
+      <c r="N7" s="13">
+        <v>188.226</v>
+      </c>
+      <c r="O7" s="13">
+        <v>0</v>
+      </c>
+      <c r="P7" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q7" s="27">
+        <v>0</v>
+      </c>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
+    </row>
+    <row r="8" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="16">
+        <v>45558</v>
+      </c>
+      <c r="D8" s="16"/>
+      <c r="E8" s="18">
+        <v>3301.6697730206133</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="9">
+        <v>34557</v>
+      </c>
+      <c r="J8" s="10">
+        <v>31</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="L8" s="12">
+        <v>984.21</v>
+      </c>
+      <c r="M8" s="12">
+        <v>787.36800000000005</v>
+      </c>
+      <c r="N8" s="13">
+        <v>196.84200000000001</v>
+      </c>
+      <c r="O8" s="13">
+        <v>0</v>
+      </c>
+      <c r="P8" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q8" s="27">
+        <v>0</v>
+      </c>
+      <c r="R8" s="28"/>
+      <c r="S8" s="28"/>
+      <c r="T8" s="28"/>
+    </row>
+    <row r="9" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="16">
+        <v>45796</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="18">
+        <v>4138.7840446837417</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="H9" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="9">
+        <v>37823</v>
+      </c>
+      <c r="J9" s="10">
+        <v>22</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="12">
+        <v>0</v>
+      </c>
+      <c r="M9" s="12">
+        <v>0</v>
+      </c>
+      <c r="N9" s="13">
+        <v>0</v>
+      </c>
+      <c r="O9" s="13">
+        <v>0</v>
+      </c>
+      <c r="P9" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="27">
+        <v>0</v>
+      </c>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28"/>
+      <c r="T9" s="28"/>
+    </row>
+    <row r="10" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="C10" s="16">
+        <v>45459</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="18">
+        <v>3304.1240295491857</v>
+      </c>
+      <c r="F10" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="G10" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="9">
+        <v>37122</v>
+      </c>
+      <c r="J10" s="10">
+        <v>24</v>
+      </c>
+      <c r="K10" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" s="12">
+        <v>0</v>
+      </c>
+      <c r="M10" s="12">
+        <v>0</v>
+      </c>
+      <c r="N10" s="13">
+        <v>0</v>
+      </c>
+      <c r="O10" s="13">
+        <v>0</v>
+      </c>
+      <c r="P10" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="27">
+        <v>0</v>
+      </c>
+      <c r="R10" s="28"/>
+      <c r="S10" s="28"/>
+      <c r="T10" s="28"/>
+    </row>
+    <row r="11" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="16">
+        <v>45894</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="18">
+        <v>4999.1267713740408</v>
+      </c>
+      <c r="F11" s="17" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="19">
-        <v>45459</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="21">
-        <v>1000</v>
-      </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="16" t="s">
+      <c r="G11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="12">
-        <v>37122</v>
-      </c>
-      <c r="K3" s="13">
-        <f ca="1">DATEDIF($J3,TODAY(),"Y")</f>
-        <v>24</v>
-      </c>
-      <c r="L3" s="22" t="str">
-        <f ca="1">IF($K3&lt;=18,"0-18",
-IF($K3&lt;=23,"19-23",
-IF($K3&lt;=28,"24-28",
-IF($K3&lt;=33,"29-33",
-IF($K3&lt;=38,"34-38",
-IF($K3&lt;=43,"39-43",
-IF($K3&lt;=48,"44-48",
-IF($K3&lt;=53,"49-53",
-IF($K3&lt;=58,"54-58","59 ou mais"
-)))))))))</f>
-        <v>24-28</v>
-      </c>
-      <c r="M3" s="15">
-        <v>0</v>
-      </c>
-      <c r="N3" s="15">
-        <f t="shared" ref="N3:N5" si="0">M3*80%</f>
-        <v>0</v>
-      </c>
-      <c r="O3" s="16">
-        <f t="shared" ref="O3:O5" si="1">M3*20%</f>
-        <v>0</v>
-      </c>
-      <c r="P3" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="16">
-        <v>0</v>
-      </c>
-      <c r="R3" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="19">
-        <v>45894</v>
-      </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="21">
-        <v>1000</v>
-      </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="16" t="s">
+      <c r="H11" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="9">
+        <v>37773</v>
+      </c>
+      <c r="J11" s="10">
         <v>22</v>
       </c>
-      <c r="J4" s="12">
-        <v>37773</v>
-      </c>
-      <c r="K4" s="13">
-        <f t="shared" ref="K3:K5" ca="1" si="2">DATEDIF(J4,TODAY(),"Y")</f>
-        <v>22</v>
-      </c>
-      <c r="L4" s="22" t="str">
-        <f t="shared" ref="L4:L5" ca="1" si="3">IF($K4&lt;=18,"0-18",
-IF($K4&lt;=23,"19-23",
-IF($K4&lt;=28,"24-28",
-IF($K4&lt;=33,"29-33",
-IF($K4&lt;=38,"34-38",
-IF($K4&lt;=43,"39-43",
-IF($K4&lt;=48,"44-48",
-IF($K4&lt;=53,"49-53",
-IF($K4&lt;=58,"54-58","59 ou mais"
-)))))))))</f>
-        <v>19-23</v>
-      </c>
-      <c r="M4" s="15">
-        <v>0</v>
-      </c>
-      <c r="N4" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O4" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P4" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="16">
-        <v>0</v>
-      </c>
-      <c r="R4" s="16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="25">
-        <v>45936</v>
-      </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26">
-        <v>1000</v>
-      </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="12">
-        <v>33330</v>
-      </c>
-      <c r="K5" s="13">
-        <f t="shared" ca="1" si="2"/>
-        <v>34</v>
-      </c>
-      <c r="L5" s="14" t="str">
-        <f t="shared" ca="1" si="3"/>
-        <v>34-38</v>
-      </c>
-      <c r="M5" s="15">
-        <v>0</v>
-      </c>
-      <c r="N5" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O5" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P5" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="16">
-        <v>0</v>
-      </c>
-      <c r="R5" s="16">
-        <v>0</v>
-      </c>
+      <c r="K11" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="L11" s="12">
+        <v>0</v>
+      </c>
+      <c r="M11" s="12">
+        <v>0</v>
+      </c>
+      <c r="N11" s="13">
+        <v>0</v>
+      </c>
+      <c r="O11" s="13">
+        <v>0</v>
+      </c>
+      <c r="P11" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="27">
+        <v>0</v>
+      </c>
+      <c r="R11" s="28"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="28"/>
+    </row>
+    <row r="17" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="24"/>
+    </row>
+    <row r="19" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="25"/>
+    </row>
+    <row r="20" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="25"/>
+    </row>
+    <row r="24" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="24"/>
+    </row>
+    <row r="27" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="25"/>
+    </row>
+    <row r="28" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="25"/>
+    </row>
+    <row r="29" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="25"/>
+    </row>
+    <row r="30" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="25"/>
+    </row>
+    <row r="31" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="25"/>
+    </row>
+    <row r="32" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>